<commit_message>
Lista atualizada com requisitos do estacionamento
2a versão da lista com requisitos identificados por pesquisa de referencias
</commit_message>
<xml_diff>
--- a/pastaDocsEngenharia/ListaDeRequisitosSiEstacionamento.xlsx
+++ b/pastaDocsEngenharia/ListaDeRequisitosSiEstacionamento.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER\Desktop\FIAP\2 PERIODO\PastaDocsEngenhariaSW\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6351EFD-B19D-4F66-A53A-5CEF3FF5F12F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75347E8F-41BD-4E4E-9585-A27B86B52587}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3585" yWindow="4995" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1170" yWindow="1170" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Plan1" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="48">
   <si>
     <t>LISTA DE REQUISITOS DO PROJETO DE SISTEMA DE INFORMAÇÃO PARA GERENCIAR ESTACIONAMENTOS</t>
   </si>
@@ -43,13 +43,142 @@
   </si>
   <si>
     <t>Descrição da Regra de domínio</t>
+  </si>
+  <si>
+    <t>Tarifação Inteligente</t>
+  </si>
+  <si>
+    <t>Rf001</t>
+  </si>
+  <si>
+    <t>Rf002</t>
+  </si>
+  <si>
+    <t>Planos Mensais</t>
+  </si>
+  <si>
+    <t>Parcerias de Convênios</t>
+  </si>
+  <si>
+    <t>Acompanhamento do caixa</t>
+  </si>
+  <si>
+    <t>Criação de anotação/lembretes</t>
+  </si>
+  <si>
+    <t>Criação de vouchers</t>
+  </si>
+  <si>
+    <t>Controle de serviços extras</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Acréscimo de serviços como lava-jato, lava-rápido, cera, polimento </t>
+  </si>
+  <si>
+    <t>Proteção do sistema com anti-fraude;</t>
+  </si>
+  <si>
+    <t>Localizar Estacionamentos Disponiveis</t>
+  </si>
+  <si>
+    <t>Reserva de vaga</t>
+  </si>
+  <si>
+    <t>Rf003</t>
+  </si>
+  <si>
+    <t>Rf004</t>
+  </si>
+  <si>
+    <t>Rf005</t>
+  </si>
+  <si>
+    <t>Rf006</t>
+  </si>
+  <si>
+    <t>Rf007</t>
+  </si>
+  <si>
+    <t>Rf008</t>
+  </si>
+  <si>
+    <t>Rf009</t>
+  </si>
+  <si>
+    <t>Rf010</t>
+  </si>
+  <si>
+    <t>Um motorista em movimento ou antes de sair com seu carro pode reservar uma vaga para um dia horario em um estacionamento</t>
+  </si>
+  <si>
+    <t>Pagamento integrado</t>
+  </si>
+  <si>
+    <t>Aceitar pagamenro com cartões ou pix</t>
+  </si>
+  <si>
+    <t>Apresentar um gráfico de barras com a quantidade de veículos por dia de um mês selecionado</t>
+  </si>
+  <si>
+    <t>Dashboard/painel de acompanhamento de ocupação por mês</t>
+  </si>
+  <si>
+    <t>Dashboard/painel de acompanhamento de receitas mês a mês</t>
+  </si>
+  <si>
+    <t>Rf011</t>
+  </si>
+  <si>
+    <t>Rf012</t>
+  </si>
+  <si>
+    <t>Rf013</t>
+  </si>
+  <si>
+    <t>Notificação de tempo restante</t>
+  </si>
+  <si>
+    <t>Com auxilio de IA, o sistema vai propor uma tarida conforme as pratica de concorentes na regiao</t>
+  </si>
+  <si>
+    <t>Tabela de preços exclusiva para mensalistas</t>
+  </si>
+  <si>
+    <t>Tabela de preços exclusiva para conveniados</t>
+  </si>
+  <si>
+    <t>Tabela de preços exclusiva para estacionamento avulso, cobrado conforme dia e horário</t>
+  </si>
+  <si>
+    <t>Registro de pagamento com controle fiscal</t>
+  </si>
+  <si>
+    <t>Apresentar um gráfico delinhas com a meses no eixo x e montante de valor recebido em R$ no eixo y</t>
+  </si>
+  <si>
+    <t>Rf014</t>
+  </si>
+  <si>
+    <t>Planos Avulsos</t>
+  </si>
+  <si>
+    <t>Rf015</t>
+  </si>
+  <si>
+    <t>Enviar Mensagem por Whatsapp para o motorista avisando o tempio restante em caso de fechamento do estacionamento</t>
+  </si>
+  <si>
+    <t>Gerar automaticamente um voucher de desconto conforme o numero de horas que o cliente acumulou em um periodo(desconto parametrizável)</t>
+  </si>
+  <si>
+    <t>Aplicação Móvel para motoristas acharem vagas de estacionamento com vagas livres na regiao em que estão, com seu preços para o horário edia</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -73,6 +202,20 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="8" tint="-0.499984740745262"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -89,12 +232,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="-0.249977111117893"/>
+        <fgColor theme="4" tint="0.39997558519241921"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="6">
+  <borders count="15">
     <border>
       <left/>
       <right/>
@@ -137,9 +280,7 @@
       <right style="thin">
         <color indexed="64"/>
       </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
+      <top/>
       <bottom style="medium">
         <color indexed="64"/>
       </bottom>
@@ -152,9 +293,7 @@
       <right style="thin">
         <color indexed="64"/>
       </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
+      <top/>
       <bottom style="medium">
         <color indexed="64"/>
       </bottom>
@@ -167,26 +306,125 @@
       <right style="medium">
         <color indexed="64"/>
       </right>
-      <top style="medium">
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
         <color indexed="64"/>
       </top>
-      <bottom style="medium">
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
         <color indexed="64"/>
       </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
       <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -470,115 +708,201 @@
   <dimension ref="A1:C20"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="91" customWidth="1"/>
-    <col min="2" max="2" width="18.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="28.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11" customWidth="1"/>
+    <col min="2" max="2" width="56.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="131.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="6"/>
-      <c r="C1" s="6"/>
+      <c r="B1" s="8"/>
+      <c r="C1" s="9"/>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" s="6" t="s">
+      <c r="A2" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="6"/>
-      <c r="C2" s="6"/>
-    </row>
-    <row r="3" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="6"/>
-      <c r="B3" s="6"/>
-      <c r="C3" s="6"/>
+      <c r="B2" s="3"/>
+      <c r="C2" s="11"/>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" s="12"/>
+      <c r="B3" s="13"/>
+      <c r="C3" s="14"/>
     </row>
     <row r="4" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="C4" s="6" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" s="2"/>
-      <c r="B5" s="2"/>
-      <c r="C5" s="2"/>
+      <c r="A5" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>36</v>
+      </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" s="1"/>
-      <c r="B6" s="1"/>
-      <c r="C6" s="1"/>
+      <c r="A6" s="15" t="s">
+        <v>7</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>37</v>
+      </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" s="1"/>
-      <c r="B7" s="1"/>
-      <c r="C7" s="1"/>
+      <c r="A7" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>38</v>
+      </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" s="1"/>
-      <c r="B8" s="1"/>
-      <c r="C8" s="1"/>
+      <c r="A8" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>40</v>
+      </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" s="1"/>
-      <c r="B9" s="1"/>
+      <c r="A9" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>11</v>
+      </c>
       <c r="C9" s="1"/>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" s="1"/>
-      <c r="B10" s="1"/>
-      <c r="C10" s="1"/>
+      <c r="A10" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>46</v>
+      </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" s="1"/>
-      <c r="B11" s="1"/>
-      <c r="C11" s="1"/>
+      <c r="A11" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" s="1"/>
-      <c r="B12" s="1"/>
+      <c r="A12" s="15" t="s">
+        <v>23</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="C12" s="1"/>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" s="1"/>
-      <c r="B13" s="1"/>
-      <c r="C13" s="1"/>
+      <c r="A13" s="15" t="s">
+        <v>24</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>47</v>
+      </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A14" s="1"/>
-      <c r="B14" s="1"/>
-      <c r="C14" s="1"/>
+      <c r="A14" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A15" s="1"/>
-      <c r="B15" s="1"/>
-      <c r="C15" s="1"/>
+      <c r="A15" s="15" t="s">
+        <v>32</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>28</v>
+      </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A16" s="1"/>
-      <c r="B16" s="1"/>
-      <c r="C16" s="1"/>
+      <c r="A16" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>29</v>
+      </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A17" s="1"/>
-      <c r="B17" s="1"/>
-      <c r="C17" s="1"/>
+      <c r="A17" s="15" t="s">
+        <v>34</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>41</v>
+      </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A18" s="1"/>
-      <c r="B18" s="1"/>
-      <c r="C18" s="1"/>
+      <c r="A18" s="15" t="s">
+        <v>42</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C18" s="16" t="s">
+        <v>45</v>
+      </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" s="1"/>
-      <c r="B19" s="1"/>
-      <c r="C19" s="1"/>
+      <c r="A19" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>39</v>
+      </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="1"/>
@@ -586,6 +910,8 @@
       <c r="C20" s="1"/>
     </row>
   </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>